<commit_message>
quartely update first run and mpi updates
</commit_message>
<xml_diff>
--- a/results/04-2026/beta/contributions-04-2026.xlsx
+++ b/results/04-2026/beta/contributions-04-2026.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -191,12 +191,12 @@
     <t xml:space="preserve">2026 Q1</t>
   </si>
   <si>
+    <t xml:space="preserve">2026 Q2</t>
+  </si>
+  <si>
     <t xml:space="preserve">projection</t>
   </si>
   <si>
-    <t xml:space="preserve">2026 Q2</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026 Q3</t>
   </si>
   <si>
@@ -213,6 +213,9 @@
   </si>
   <si>
     <t xml:space="preserve">2027 Q4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2028 Q1</t>
   </si>
 </sst>
 </file>
@@ -2994,7 +2997,7 @@
         <v>0.142483137788292</v>
       </c>
       <c r="J25" t="n">
-        <v>0.0187005366381567</v>
+        <v>0.00840005838598947</v>
       </c>
       <c r="K25" t="n">
         <v>0.137992081379504</v>
@@ -3027,7 +3030,7 @@
         <v>-0.0076726144240776</v>
       </c>
       <c r="U25" t="n">
-        <v>-0.0242890509138495</v>
+        <v>-0.0242646124776583</v>
       </c>
       <c r="V25" t="n">
         <v>-0.0000531438557844164</v>
@@ -3045,25 +3048,25 @@
         <v>0.272737134010574</v>
       </c>
       <c r="AA25" t="n">
-        <v>-0.259838890856755</v>
+        <v>-0.270169588737866</v>
       </c>
       <c r="AB25" t="n">
-        <v>0.329022042419087</v>
+        <v>0.329046389863244</v>
       </c>
       <c r="AC25" t="n">
-        <v>0.0700839628014538</v>
+        <v>0.0598134793214488</v>
       </c>
       <c r="AD25" t="n">
-        <v>-0.402322028645047</v>
+        <v>-0.412652726526158</v>
       </c>
       <c r="AE25" t="n">
-        <v>0.353311093332936</v>
+        <v>0.353311002340902</v>
       </c>
       <c r="AF25" t="n">
-        <v>-1.24765869997213</v>
+        <v>-1.25792918345213</v>
       </c>
       <c r="AG25" t="n">
-        <v>-0.528896712382591</v>
+        <v>-0.531464333252592</v>
       </c>
     </row>
     <row r="26">
@@ -3071,138 +3074,138 @@
         <v>58</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D26" t="n">
-        <v>1.66614404825135</v>
+        <v>0.436508484478446</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.188704745478899</v>
+        <v>-0.0710580054369052</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.0227340968335049</v>
+        <v>0.0501880171233495</v>
       </c>
       <c r="G26" t="n">
-        <v>0.028247717760595</v>
+        <v>0.0586159262003014</v>
       </c>
       <c r="H26" t="n">
-        <v>0.0230908327045624</v>
+        <v>0.0274466981777993</v>
       </c>
       <c r="I26" t="n">
-        <v>0.313134521728542</v>
+        <v>0.314515777091386</v>
       </c>
       <c r="J26" t="n">
-        <v>0.0167727057307057</v>
+        <v>0.0132072895661503</v>
       </c>
       <c r="K26" t="n">
-        <v>-0.0399401532635637</v>
+        <v>-0.226200693276775</v>
       </c>
       <c r="L26" t="n">
-        <v>0.0328468378633532</v>
+        <v>-0.0403316913163063</v>
       </c>
       <c r="M26" t="n">
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>-0.000947267993169992</v>
+        <v>-0.000960782164182661</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
       <c r="P26" t="n">
-        <v>-0.0102942452796516</v>
+        <v>-0.00908597075489488</v>
       </c>
       <c r="Q26" t="n">
-        <v>-0.019590885584065</v>
+        <v>0.00411399790277102</v>
       </c>
       <c r="R26" t="n">
-        <v>-0.00268390951436379</v>
+        <v>-0.00273081610851882</v>
       </c>
       <c r="S26" t="n">
-        <v>-0.0143869288496247</v>
+        <v>-0.0146408228761549</v>
       </c>
       <c r="T26" t="n">
-        <v>-0.00710978917847009</v>
+        <v>-0.00724609284152218</v>
       </c>
       <c r="U26" t="n">
-        <v>-0.0223516886372291</v>
+        <v>-0.00125291743599055</v>
       </c>
       <c r="V26" t="n">
-        <v>-0.000517122684655328</v>
+        <v>-0.0000696617484409661</v>
       </c>
       <c r="W26" t="n">
-        <v>0.22476206195789</v>
+        <v>0.224985702190415</v>
       </c>
       <c r="X26" t="n">
-        <v>0.0229002032225388</v>
+        <v>0.0124692193307716</v>
       </c>
       <c r="Y26" t="n">
-        <v>1.61468392753924</v>
+        <v>0.299681722190402</v>
       </c>
       <c r="Z26" t="n">
-        <v>-0.137244624766788</v>
+        <v>0.0657687568511386</v>
       </c>
       <c r="AA26" t="n">
-        <v>0.358361790668108</v>
+        <v>0.463404670727734</v>
       </c>
       <c r="AB26" t="n">
-        <v>0.162837776260205</v>
+        <v>-0.0604293144674622</v>
       </c>
       <c r="AC26" t="n">
-        <v>0.580582306938243</v>
+        <v>0.463266623529774</v>
       </c>
       <c r="AD26" t="n">
-        <v>0.0452272689395654</v>
+        <v>0.148888893636348</v>
       </c>
       <c r="AE26" t="n">
-        <v>0.185189464897434</v>
+        <v>-0.0591763970314716</v>
       </c>
       <c r="AF26" t="n">
-        <v>2.05802160971069</v>
+        <v>0.828717102571314</v>
       </c>
       <c r="AG26" t="n">
-        <v>0.159372108311035</v>
+        <v>-0.15052163934381</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27" t="s">
         <v>60</v>
       </c>
-      <c r="B27" t="s">
-        <v>59</v>
-      </c>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.420709831037319</v>
+        <v>-0.246043988517862</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.176184247400425</v>
+        <v>-0.177384890887503</v>
       </c>
       <c r="F27" t="n">
-        <v>-0.0565006293763161</v>
+        <v>-0.0187909592274629</v>
       </c>
       <c r="G27" t="n">
-        <v>-0.00880150241652977</v>
+        <v>-0.0135823615948663</v>
       </c>
       <c r="H27" t="n">
-        <v>0.020506223308859</v>
+        <v>0.0204825031770616</v>
       </c>
       <c r="I27" t="n">
-        <v>0.251833673563064</v>
+        <v>0.25154363993049</v>
       </c>
       <c r="J27" t="n">
-        <v>0.0123004390178763</v>
+        <v>0.0070302754234444</v>
       </c>
       <c r="K27" t="n">
-        <v>-0.18964298329505</v>
+        <v>-0.281581188453789</v>
       </c>
       <c r="L27" t="n">
-        <v>0.0473865174312755</v>
+        <v>0.0481548133569815</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
@@ -3214,58 +3217,58 @@
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>-0.00899748036153736</v>
+        <v>-0.00932521182800695</v>
       </c>
       <c r="Q27" t="n">
-        <v>-0.0144565211050625</v>
+        <v>0.00643770175100916</v>
       </c>
       <c r="R27" t="n">
-        <v>-0.00223770188924322</v>
+        <v>-0.00223511236832679</v>
       </c>
       <c r="S27" t="n">
-        <v>-0.00983310836289468</v>
+        <v>-0.00982172763539681</v>
       </c>
       <c r="T27" t="n">
-        <v>-0.00646591694202064</v>
+        <v>-0.00645843383716623</v>
       </c>
       <c r="U27" t="n">
-        <v>-0.0205297639592623</v>
+        <v>-0.00308365752099749</v>
       </c>
       <c r="V27" t="n">
-        <v>-0.000434869020035866</v>
+        <v>-0.000501429966115183</v>
       </c>
       <c r="W27" t="n">
-        <v>0.214079581465423</v>
+        <v>0.207022102238222</v>
       </c>
       <c r="X27" t="n">
-        <v>0.0322655618445932</v>
+        <v>0.0365288260044681</v>
       </c>
       <c r="Y27" t="n">
-        <v>-0.505498412760509</v>
+        <v>-0.330545226387455</v>
       </c>
       <c r="Z27" t="n">
-        <v>-0.0913956656772347</v>
+        <v>-0.0928836530179101</v>
       </c>
       <c r="AA27" t="n">
-        <v>0.219438889884077</v>
+        <v>0.246701059341931</v>
       </c>
       <c r="AB27" t="n">
-        <v>0.0415761599621467</v>
+        <v>-0.0142040674807482</v>
       </c>
       <c r="AC27" t="n">
-        <v>0.320919075194145</v>
+        <v>0.292533742073643</v>
       </c>
       <c r="AD27" t="n">
-        <v>-0.0323947836789873</v>
+        <v>-0.00484258058855852</v>
       </c>
       <c r="AE27" t="n">
-        <v>0.0621059239214089</v>
+        <v>-0.0111204099597507</v>
       </c>
       <c r="AF27" t="n">
-        <v>-0.275975003243598</v>
+        <v>-0.130895137331722</v>
       </c>
       <c r="AG27" t="n">
-        <v>0.198675708464536</v>
+        <v>-0.0749480727123405</v>
       </c>
     </row>
     <row r="28">
@@ -3273,37 +3276,37 @@
         <v>61</v>
       </c>
       <c r="B28" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.150858146592394</v>
+        <v>-0.146342913256379</v>
       </c>
       <c r="E28" t="n">
-        <v>-0.175043552790665</v>
+        <v>-0.176236422781678</v>
       </c>
       <c r="F28" t="n">
-        <v>-0.109557240622333</v>
+        <v>-0.0755164154931463</v>
       </c>
       <c r="G28" t="n">
-        <v>-0.0116662370392203</v>
+        <v>-0.0140897876009744</v>
       </c>
       <c r="H28" t="n">
-        <v>0.0304195921974103</v>
+        <v>0.0303844116342299</v>
       </c>
       <c r="I28" t="n">
-        <v>0.0780207605778426</v>
+        <v>0.0779306099692082</v>
       </c>
       <c r="J28" t="n">
-        <v>0.0108989230434262</v>
+        <v>0.00575040802720318</v>
       </c>
       <c r="K28" t="n">
-        <v>-0.00546385491572805</v>
+        <v>-0.0949762773294562</v>
       </c>
       <c r="L28" t="n">
-        <v>0.0544809327441534</v>
+        <v>0.0552129718663187</v>
       </c>
       <c r="M28" t="n">
         <v>0</v>
@@ -3315,58 +3318,58 @@
         <v>0</v>
       </c>
       <c r="P28" t="n">
-        <v>-0.00970680057072466</v>
+        <v>-0.0098190376523815</v>
       </c>
       <c r="Q28" t="n">
-        <v>-0.0126215734177798</v>
+        <v>0.00661357997019864</v>
       </c>
       <c r="R28" t="n">
-        <v>-0.00281262448770808</v>
+        <v>-0.00280936961711405</v>
       </c>
       <c r="S28" t="n">
-        <v>-0.00668782996714076</v>
+        <v>-0.00668009000270352</v>
       </c>
       <c r="T28" t="n">
-        <v>-0.00574772632456763</v>
+        <v>-0.00574107447962623</v>
       </c>
       <c r="U28" t="n">
-        <v>-0.019447025589517</v>
+        <v>0.00426063987336252</v>
       </c>
       <c r="V28" t="n">
-        <v>-0.000402619731988997</v>
+        <v>-0.000426940925803921</v>
       </c>
       <c r="W28" t="n">
-        <v>0.170716249234254</v>
+        <v>0.162770134174828</v>
       </c>
       <c r="X28" t="n">
-        <v>-0.0297158643115744</v>
+        <v>-0.0273950236581683</v>
       </c>
       <c r="Y28" t="n">
-        <v>-0.187456851853127</v>
+        <v>-0.182706291067979</v>
       </c>
       <c r="Z28" t="n">
-        <v>-0.138444847529932</v>
+        <v>-0.139873044970078</v>
       </c>
       <c r="AA28" t="n">
-        <v>-0.00178253435925942</v>
+        <v>0.0245241152126061</v>
       </c>
       <c r="AB28" t="n">
-        <v>0.132676576504906</v>
+        <v>0.0811831420485551</v>
       </c>
       <c r="AC28" t="n">
-        <v>0.190896539488912</v>
+        <v>0.165686297543363</v>
       </c>
       <c r="AD28" t="n">
-        <v>-0.079803294937102</v>
+        <v>-0.0534064947566021</v>
       </c>
       <c r="AE28" t="n">
-        <v>0.152123602094423</v>
+        <v>0.0769225021751926</v>
       </c>
       <c r="AF28" t="n">
-        <v>-0.135005159894147</v>
+        <v>-0.156893038494693</v>
       </c>
       <c r="AG28" t="n">
-        <v>0.099845686650204</v>
+        <v>-0.179250064176809</v>
       </c>
     </row>
     <row r="29">
@@ -3374,37 +3377,37 @@
         <v>62</v>
       </c>
       <c r="B29" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.110173388408814</v>
+        <v>-0.10687586310228</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.198593458052039</v>
+        <v>-0.199946813675512</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.0938691318649901</v>
+        <v>-0.0755269715214324</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.00721340500497764</v>
+        <v>-0.00902915102977396</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0272401105490608</v>
+        <v>0.0272086052503855</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.0523522549602245</v>
+        <v>-0.0522916142007128</v>
       </c>
       <c r="J29" t="n">
-        <v>0.0116792142668356</v>
+        <v>0.00661876362926851</v>
       </c>
       <c r="K29" t="n">
-        <v>0.0351930300938164</v>
+        <v>-0.0521551690697122</v>
       </c>
       <c r="L29" t="n">
-        <v>0.0589448427500478</v>
+        <v>0.0596308122823412</v>
       </c>
       <c r="M29" t="n">
         <v>0</v>
@@ -3416,58 +3419,58 @@
         <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>-0.00922620457866887</v>
+        <v>-0.00933535606876166</v>
       </c>
       <c r="Q29" t="n">
-        <v>-0.00855857232959935</v>
+        <v>0.00912133714131898</v>
       </c>
       <c r="R29" t="n">
-        <v>-0.000293382507181051</v>
+        <v>-0.000293043010447602</v>
       </c>
       <c r="S29" t="n">
-        <v>-0.00303213847028566</v>
+        <v>-0.00302862955485382</v>
       </c>
       <c r="T29" t="n">
-        <v>-0.0031681598427723</v>
+        <v>-0.00316449350844382</v>
       </c>
       <c r="U29" t="n">
-        <v>-0.0123226453887189</v>
+        <v>0.00863155222093056</v>
       </c>
       <c r="V29" t="n">
-        <v>-0.000371559930609723</v>
+        <v>-0.000395175505607586</v>
       </c>
       <c r="W29" t="n">
-        <v>0.116915450722698</v>
+        <v>0.110104285704918</v>
       </c>
       <c r="X29" t="n">
-        <v>-0.0152025009432854</v>
+        <v>-0.0142421131305181</v>
       </c>
       <c r="Y29" t="n">
-        <v>-0.169527870704099</v>
+        <v>-0.165982905043573</v>
       </c>
       <c r="Z29" t="n">
-        <v>-0.139238975756754</v>
+        <v>-0.140839771734219</v>
       </c>
       <c r="AA29" t="n">
-        <v>-0.11451878982377</v>
+        <v>-0.103027263284356</v>
       </c>
       <c r="AB29" t="n">
-        <v>0.158844757937732</v>
+        <v>0.104915517060876</v>
       </c>
       <c r="AC29" t="n">
-        <v>0.104518673248615</v>
+        <v>0.0620024107926297</v>
       </c>
       <c r="AD29" t="n">
-        <v>-0.0621665348635455</v>
+        <v>-0.0507356490836435</v>
       </c>
       <c r="AE29" t="n">
-        <v>0.171167403326451</v>
+        <v>0.0962839648399452</v>
       </c>
       <c r="AF29" t="n">
-        <v>-0.204248173212239</v>
+        <v>-0.244820265985162</v>
       </c>
       <c r="AG29" t="n">
-        <v>0.360698318340177</v>
+        <v>0.0740271651899341</v>
       </c>
     </row>
     <row r="30">
@@ -3475,37 +3478,37 @@
         <v>63</v>
       </c>
       <c r="B30" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.11749209491152</v>
+        <v>-0.11397551834177</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.184954364701993</v>
+        <v>-0.186214773942108</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.346033074678445</v>
+        <v>-0.344016665038198</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.00701225480204403</v>
+        <v>-0.00871948653904214</v>
       </c>
       <c r="H30" t="n">
-        <v>0.0370277067636871</v>
+        <v>0.0369848894040224</v>
       </c>
       <c r="I30" t="n">
-        <v>-0.267184694661036</v>
+        <v>-0.266873947521892</v>
       </c>
       <c r="J30" t="n">
-        <v>0.0117504457810699</v>
+        <v>0.00682585935486931</v>
       </c>
       <c r="K30" t="n">
-        <v>0.0295327400207467</v>
+        <v>0.0447272629054179</v>
       </c>
       <c r="L30" t="n">
-        <v>0.00839718520675031</v>
+        <v>0.0741760058200484</v>
       </c>
       <c r="M30" t="n">
         <v>0</v>
@@ -3517,58 +3520,58 @@
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>-0.00442812281376111</v>
+        <v>-0.00503959208748433</v>
       </c>
       <c r="Q30" t="n">
-        <v>-0.00792813540768285</v>
+        <v>0.00719311552019024</v>
       </c>
       <c r="R30" t="n">
-        <v>-0.000286302962534931</v>
+        <v>-0.000285971658178611</v>
       </c>
       <c r="S30" t="n">
-        <v>-0.00134832978737942</v>
+        <v>-0.00134676949436724</v>
       </c>
       <c r="T30" t="n">
-        <v>-0.00178157103577599</v>
+        <v>-0.00177950937707208</v>
       </c>
       <c r="U30" t="n">
-        <v>-0.011697636380997</v>
+        <v>0.00237422153404077</v>
       </c>
       <c r="V30" t="n">
-        <v>-0.000322956686060288</v>
+        <v>-0.000365697253103981</v>
       </c>
       <c r="W30" t="n">
-        <v>0.114722443042679</v>
+        <v>0.0747419360682316</v>
       </c>
       <c r="X30" t="n">
-        <v>-0.00711649746668697</v>
+        <v>-0.00432257924151644</v>
       </c>
       <c r="Y30" t="n">
-        <v>-0.163987462838498</v>
+        <v>-0.1602387861888</v>
       </c>
       <c r="Z30" t="n">
-        <v>-0.138458996775016</v>
+        <v>-0.139951506095078</v>
       </c>
       <c r="AA30" t="n">
-        <v>-0.572162185606492</v>
+        <v>-0.576542611312116</v>
       </c>
       <c r="AB30" t="n">
-        <v>0.117745548833549</v>
+        <v>0.18995088856399</v>
       </c>
       <c r="AC30" t="n">
-        <v>-0.39370107053356</v>
+        <v>-0.325431845805402</v>
       </c>
       <c r="AD30" t="n">
-        <v>-0.304977490945456</v>
+        <v>-0.309668663790224</v>
       </c>
       <c r="AE30" t="n">
-        <v>0.129443185214546</v>
+        <v>0.187576667029949</v>
       </c>
       <c r="AF30" t="n">
-        <v>-0.696147530147073</v>
+        <v>-0.62562213808928</v>
       </c>
       <c r="AG30" t="n">
-        <v>-0.327843966624264</v>
+        <v>-0.289557644975215</v>
       </c>
     </row>
     <row r="31">
@@ -3576,37 +3579,37 @@
         <v>64</v>
       </c>
       <c r="B31" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.100537913769166</v>
+        <v>-0.0975287813488231</v>
       </c>
       <c r="E31" t="n">
-        <v>-0.179518090858253</v>
+        <v>-0.18074145350152</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.20875387886039</v>
+        <v>-0.206803941679915</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.00274072405671313</v>
+        <v>-0.00433211445750534</v>
       </c>
       <c r="H31" t="n">
-        <v>0.0438384716842681</v>
+        <v>0.043787785295544</v>
       </c>
       <c r="I31" t="n">
-        <v>-0.364246832230586</v>
+        <v>-0.36382241629954</v>
       </c>
       <c r="J31" t="n">
-        <v>0.0103326017155023</v>
+        <v>0.00551495121579593</v>
       </c>
       <c r="K31" t="n">
-        <v>0.0366137137752495</v>
+        <v>0.0136782857117134</v>
       </c>
       <c r="L31" t="n">
-        <v>0.00890406050198482</v>
+        <v>0.00889375869671701</v>
       </c>
       <c r="M31" t="n">
         <v>0</v>
@@ -3618,58 +3621,58 @@
         <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>-0.00142312480846168</v>
+        <v>-0.00182656494149161</v>
       </c>
       <c r="Q31" t="n">
-        <v>-0.00805673466147888</v>
+        <v>0.00673218956558858</v>
       </c>
       <c r="R31" t="n">
-        <v>-0.000279932204496591</v>
+        <v>-0.000279608272315239</v>
       </c>
       <c r="S31" t="n">
-        <v>-0.00101864471012829</v>
+        <v>-0.00101746593741716</v>
       </c>
       <c r="T31" t="n">
-        <v>-0.00149913524971762</v>
+        <v>-0.00149740043885975</v>
       </c>
       <c r="U31" t="n">
-        <v>-0.00978076307697897</v>
+        <v>-0.000323854182184991</v>
       </c>
       <c r="V31" t="n">
-        <v>-0.000315600107555253</v>
+        <v>-0.000318458448563437</v>
       </c>
       <c r="W31" t="n">
-        <v>0.0616095842025686</v>
+        <v>0.0602243053891414</v>
       </c>
       <c r="X31" t="n">
-        <v>-0.0109793532176722</v>
+        <v>-0.0135877228904138</v>
       </c>
       <c r="Y31" t="n">
-        <v>-0.145311068813816</v>
+        <v>-0.14208312752099</v>
       </c>
       <c r="Z31" t="n">
-        <v>-0.134744935813603</v>
+        <v>-0.136187107329353</v>
       </c>
       <c r="AA31" t="n">
-        <v>-0.522068802934925</v>
+        <v>-0.526181744940237</v>
       </c>
       <c r="AB31" t="n">
-        <v>0.0737743822701202</v>
+        <v>0.0706728660628411</v>
       </c>
       <c r="AC31" t="n">
-        <v>-0.387884392606698</v>
+        <v>-0.395114181789943</v>
       </c>
       <c r="AD31" t="n">
-        <v>-0.157821970704339</v>
+        <v>-0.162359328640697</v>
       </c>
       <c r="AE31" t="n">
-        <v>0.0835551453470992</v>
+        <v>0.0709967202450261</v>
       </c>
       <c r="AF31" t="n">
-        <v>-0.667940397234117</v>
+        <v>-0.673384416640286</v>
       </c>
       <c r="AG31" t="n">
-        <v>-0.425835315121894</v>
+        <v>-0.425179964802355</v>
       </c>
     </row>
     <row r="32">
@@ -3677,37 +3680,37 @@
         <v>65</v>
       </c>
       <c r="B32" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.107368263247405</v>
+        <v>-0.104154696248239</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.186750757530558</v>
+        <v>-0.188023408655981</v>
       </c>
       <c r="F32" t="n">
-        <v>0.0304640223038154</v>
+        <v>0.0402363932732792</v>
       </c>
       <c r="G32" t="n">
-        <v>0.000540224260864334</v>
+        <v>-0.000926599399724825</v>
       </c>
       <c r="H32" t="n">
-        <v>0.0392841583391929</v>
+        <v>0.0392387337096022</v>
       </c>
       <c r="I32" t="n">
-        <v>-0.386880253005743</v>
+        <v>-0.386429275379733</v>
       </c>
       <c r="J32" t="n">
-        <v>0.00998641367971701</v>
+        <v>0.00526846990965778</v>
       </c>
       <c r="K32" t="n">
-        <v>0.0380736733973169</v>
+        <v>0.0155719571102066</v>
       </c>
       <c r="L32" t="n">
-        <v>0.00935610800823099</v>
+        <v>0.00934528328550894</v>
       </c>
       <c r="M32" t="n">
         <v>0</v>
@@ -3719,58 +3722,58 @@
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>0.000358589023948943</v>
+        <v>0.000352838956830397</v>
       </c>
       <c r="Q32" t="n">
-        <v>-0.00827285943507663</v>
+        <v>0.00623065664900438</v>
       </c>
       <c r="R32" t="n">
-        <v>-0.000274482203485652</v>
+        <v>-0.000274164577999679</v>
       </c>
       <c r="S32" t="n">
-        <v>-0.00100236810299272</v>
+        <v>-0.00100120816583779</v>
       </c>
       <c r="T32" t="n">
-        <v>-0.00123904489460494</v>
+        <v>-0.00123761106939872</v>
       </c>
       <c r="U32" t="n">
-        <v>0.024935854277618</v>
+        <v>0.00503738545094546</v>
       </c>
       <c r="V32" t="n">
-        <v>-0.000309363502687192</v>
+        <v>-0.000312156590467466</v>
       </c>
       <c r="W32" t="n">
-        <v>0.009435814340737</v>
+        <v>0.0092716635034082</v>
       </c>
       <c r="X32" t="n">
-        <v>-0.0222591298571621</v>
+        <v>-0.0234751031805249</v>
       </c>
       <c r="Y32" t="n">
-        <v>-0.150436010658066</v>
+        <v>-0.147016752572777</v>
       </c>
       <c r="Z32" t="n">
-        <v>-0.143683010119898</v>
+        <v>-0.145161352331443</v>
       </c>
       <c r="AA32" t="n">
-        <v>-0.306295695814262</v>
+        <v>-0.302289141760856</v>
       </c>
       <c r="AB32" t="n">
-        <v>0.0488050922305394</v>
+        <v>0.0195130068435475</v>
       </c>
       <c r="AC32" t="n">
-        <v>-0.257331537250197</v>
+        <v>-0.282713560069184</v>
       </c>
       <c r="AD32" t="n">
-        <v>0.0805845571914808</v>
+        <v>0.0841401336188763</v>
       </c>
       <c r="AE32" t="n">
-        <v>0.0238692379529214</v>
+        <v>0.014475621392602</v>
       </c>
       <c r="AF32" t="n">
-        <v>-0.551450558028161</v>
+        <v>-0.574891664973404</v>
       </c>
       <c r="AG32" t="n">
-        <v>-0.529946664655398</v>
+        <v>-0.529679621422033</v>
       </c>
     </row>
     <row r="33">
@@ -3778,37 +3781,37 @@
         <v>66</v>
       </c>
       <c r="B33" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C33" t="n">
         <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.177302710484615</v>
+        <v>-0.171995982760397</v>
       </c>
       <c r="E33" t="n">
-        <v>-0.183246646150979</v>
+        <v>-0.184495417794735</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0689203379959541</v>
+        <v>0.0785880651114898</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0120712992194414</v>
+        <v>0.0107213802706063</v>
       </c>
       <c r="H33" t="n">
-        <v>0.0439677222278218</v>
+        <v>0.0439168865394133</v>
       </c>
       <c r="I33" t="n">
-        <v>-0.429217694598965</v>
+        <v>-0.42871696202656</v>
       </c>
       <c r="J33" t="n">
-        <v>0.0109394892890476</v>
+        <v>0.00628379817755373</v>
       </c>
       <c r="K33" t="n">
-        <v>0.00242889478013606</v>
+        <v>-0.0195741899100774</v>
       </c>
       <c r="L33" t="n">
-        <v>0.00976637754758537</v>
+        <v>0.00975507824660246</v>
       </c>
       <c r="M33" t="n">
         <v>0</v>
@@ -3820,58 +3823,159 @@
         <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>0.00259276018795545</v>
+        <v>0.00248763586780503</v>
       </c>
       <c r="Q33" t="n">
-        <v>-0.00564681216626738</v>
+        <v>0.0085490132088127</v>
       </c>
       <c r="R33" t="n">
-        <v>0.000198529911872401</v>
+        <v>0.000198300178911062</v>
       </c>
       <c r="S33" t="n">
-        <v>-0.000993960416273958</v>
+        <v>-0.000992810208750326</v>
       </c>
       <c r="T33" t="n">
-        <v>-0.000240277831537949</v>
+        <v>-0.000239999786936005</v>
       </c>
       <c r="U33" t="n">
-        <v>0.0218518238394764</v>
+        <v>0.00394094650479018</v>
       </c>
       <c r="V33" t="n">
-        <v>-0.000302765050606375</v>
+        <v>-0.000305491844496977</v>
       </c>
       <c r="W33" t="n">
-        <v>-0.00291588534563375</v>
+        <v>-0.00136295384642158</v>
       </c>
       <c r="X33" t="n">
-        <v>-0.0121918619904309</v>
+        <v>-0.0115869753952157</v>
       </c>
       <c r="Y33" t="n">
-        <v>-0.218931602374652</v>
+        <v>-0.213430042513555</v>
       </c>
       <c r="Z33" t="n">
-        <v>-0.141617754260942</v>
+        <v>-0.143061358041577</v>
       </c>
       <c r="AA33" t="n">
-        <v>-0.292759150299271</v>
+        <v>-0.288631397605301</v>
       </c>
       <c r="AB33" t="n">
-        <v>0.0145498294332267</v>
+        <v>-0.00912811548088149</v>
       </c>
       <c r="AC33" t="n">
-        <v>-0.278163943760303</v>
+        <v>-0.297787495062336</v>
       </c>
       <c r="AD33" t="n">
-        <v>0.136458544299694</v>
+        <v>0.140085564421258</v>
       </c>
       <c r="AE33" t="n">
-        <v>-0.00730199440624964</v>
+        <v>-0.0130690619856717</v>
       </c>
       <c r="AF33" t="n">
-        <v>-0.638713300395896</v>
+        <v>-0.654278895617468</v>
       </c>
       <c r="AG33" t="n">
-        <v>-0.638562946451312</v>
+        <v>-0.63204427883011</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>-0.205141427200942</v>
+      </c>
+      <c r="E34" t="n">
+        <v>-0.183578043716544</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-0.0638321272933333</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.00704988013781239</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.0255593448966518</v>
+      </c>
+      <c r="I34" t="n">
+        <v>-0.616876171778661</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.0103444268268873</v>
+      </c>
+      <c r="K34" t="n">
+        <v>-0.0919261259634657</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0.0101430800572218</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0.00208389012354234</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0.00342021698030483</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0.000194363861199969</v>
+      </c>
+      <c r="S34" t="n">
+        <v>-0.000995798705676766</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" t="n">
+        <v>0</v>
+      </c>
+      <c r="V34" t="n">
+        <v>-0.000299428155345378</v>
+      </c>
+      <c r="W34" t="n">
+        <v>-0.0331773637149976</v>
+      </c>
+      <c r="X34" t="n">
+        <v>0.00776152455226643</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>-0.245538348742651</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>-0.143181122174836</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>-0.637867527197291</v>
+      </c>
+      <c r="AB34" t="n">
+        <v>-0.10280007135667</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>-0.741363232310278</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>-0.0209913554186304</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>-0.10280007135667</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>-1.13008270322776</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>-0.758159420114731</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes to corporate taxes
added in add factors to taxes to reflect the changes to tariffs.
also includes the first round of no_tariffs and no_obbba work for the breakdown sheet, but those will have to be redone.
</commit_message>
<xml_diff>
--- a/results/04-2026/beta/contributions-04-2026.xlsx
+++ b/results/04-2026/beta/contributions-04-2026.xlsx
@@ -2884,7 +2884,7 @@
         <v>-0.0289055700739013</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.117350200113337</v>
+        <v>-0.499897395595688</v>
       </c>
       <c r="G24" t="n">
         <v>-0.014530714174193</v>
@@ -2947,25 +2947,25 @@
         <v>-0.261464773606026</v>
       </c>
       <c r="AA24" t="n">
-        <v>0.241898475197163</v>
+        <v>-0.139229581720164</v>
       </c>
       <c r="AB24" t="n">
         <v>0.400833075000047</v>
       </c>
       <c r="AC24" t="n">
-        <v>0.641727532450867</v>
+        <v>0.262180996866793</v>
       </c>
       <c r="AD24" t="n">
-        <v>0.00796655275845429</v>
+        <v>-0.373161504158873</v>
       </c>
       <c r="AE24" t="n">
         <v>0.430588072018699</v>
       </c>
       <c r="AF24" t="n">
-        <v>0.639861462947255</v>
+        <v>0.26031492736318</v>
       </c>
       <c r="AG24" t="n">
-        <v>0.00573571057558156</v>
+        <v>-0.089150923320437</v>
       </c>
     </row>
     <row r="25">
@@ -2985,7 +2985,7 @@
         <v>-0.0733698868603123</v>
       </c>
       <c r="F25" t="n">
-        <v>0.013033349568796</v>
+        <v>-0.403643992985071</v>
       </c>
       <c r="G25" t="n">
         <v>-0.030262516077315</v>
@@ -3048,25 +3048,25 @@
         <v>0.272737134010574</v>
       </c>
       <c r="AA25" t="n">
-        <v>0.145924562447469</v>
+        <v>-0.270169588737866</v>
       </c>
       <c r="AB25" t="n">
         <v>0.329046389863244</v>
       </c>
       <c r="AC25" t="n">
-        <v>0.47446466261275</v>
+        <v>0.0598134793214488</v>
       </c>
       <c r="AD25" t="n">
-        <v>0.00344142465917663</v>
+        <v>-0.412652726526158</v>
       </c>
       <c r="AE25" t="n">
         <v>0.353311002340902</v>
       </c>
       <c r="AF25" t="n">
-        <v>-0.843278000160834</v>
+        <v>-1.25792918345213</v>
       </c>
       <c r="AG25" t="n">
-        <v>-0.332914903533748</v>
+        <v>-0.531464333252592</v>
       </c>
     </row>
     <row r="26">
@@ -3086,7 +3086,7 @@
         <v>-0.0710580054369052</v>
       </c>
       <c r="F26" t="n">
-        <v>0.239406622639966</v>
+        <v>0.0501880171233495</v>
       </c>
       <c r="G26" t="n">
         <v>0.0586159262003014</v>
@@ -3149,25 +3149,25 @@
         <v>0.0657687568511386</v>
       </c>
       <c r="AA26" t="n">
-        <v>0.651809176738972</v>
+        <v>0.463404670727734</v>
       </c>
       <c r="AB26" t="n">
         <v>-0.0604293144674622</v>
       </c>
       <c r="AC26" t="n">
-        <v>0.651789683360029</v>
+        <v>0.463266623529774</v>
       </c>
       <c r="AD26" t="n">
-        <v>0.337293399647586</v>
+        <v>0.148888893636348</v>
       </c>
       <c r="AE26" t="n">
         <v>-0.0591763970314716</v>
       </c>
       <c r="AF26" t="n">
-        <v>1.01724016240157</v>
+        <v>0.828717102571314</v>
       </c>
       <c r="AG26" t="n">
-        <v>0.0951585553325976</v>
+        <v>-0.15052163934381</v>
       </c>
     </row>
     <row r="27">
@@ -3187,13 +3187,13 @@
         <v>-0.177384890887503</v>
       </c>
       <c r="F27" t="n">
-        <v>0.145349181392773</v>
+        <v>0.0906545813014853</v>
       </c>
       <c r="G27" t="n">
         <v>-0.0135823615948663</v>
       </c>
       <c r="H27" t="n">
-        <v>0.0204825031770616</v>
+        <v>0.0530552985300118</v>
       </c>
       <c r="I27" t="n">
         <v>0.25154363993049</v>
@@ -3250,25 +3250,25 @@
         <v>-0.0928836530179101</v>
       </c>
       <c r="AA27" t="n">
-        <v>0.410384135092492</v>
+        <v>0.388300039888712</v>
       </c>
       <c r="AB27" t="n">
         <v>-0.0142040674807482</v>
       </c>
       <c r="AC27" t="n">
-        <v>0.456241218675884</v>
+        <v>0.434153830494396</v>
       </c>
       <c r="AD27" t="n">
-        <v>0.158840495162002</v>
+        <v>0.136756399958222</v>
       </c>
       <c r="AE27" t="n">
         <v>-0.0111204099597507</v>
       </c>
       <c r="AF27" t="n">
-        <v>0.0328123392705189</v>
+        <v>0.0107249510890314</v>
       </c>
       <c r="AG27" t="n">
-        <v>0.211658991114627</v>
+        <v>-0.0395430506071521</v>
       </c>
     </row>
     <row r="28">
@@ -3288,13 +3288,13 @@
         <v>-0.176236422781678</v>
       </c>
       <c r="F28" t="n">
-        <v>0.102231761871102</v>
+        <v>0.0320613916729151</v>
       </c>
       <c r="G28" t="n">
         <v>-0.0140897876009744</v>
       </c>
       <c r="H28" t="n">
-        <v>0.0303844116342299</v>
+        <v>0.0611887191445801</v>
       </c>
       <c r="I28" t="n">
         <v>0.0779306099692082</v>
@@ -3351,25 +3351,25 @@
         <v>-0.139873044970078</v>
       </c>
       <c r="AA28" t="n">
-        <v>0.202085233703639</v>
+        <v>0.162760065763167</v>
       </c>
       <c r="AB28" t="n">
         <v>0.0811831420485551</v>
       </c>
       <c r="AC28" t="n">
-        <v>0.343095608249406</v>
+        <v>0.303804069949841</v>
       </c>
       <c r="AD28" t="n">
-        <v>0.12415462373443</v>
+        <v>0.0848294557939591</v>
       </c>
       <c r="AE28" t="n">
         <v>0.0769225021751926</v>
       </c>
       <c r="AF28" t="n">
-        <v>0.0205162722113488</v>
+        <v>-0.0187752660882153</v>
       </c>
       <c r="AG28" t="n">
-        <v>0.0568226934306508</v>
+        <v>-0.109315598970001</v>
       </c>
     </row>
     <row r="29">
@@ -3389,13 +3389,13 @@
         <v>-0.199946813675512</v>
       </c>
       <c r="F29" t="n">
-        <v>0.101672286414703</v>
+        <v>-0.0227724580374239</v>
       </c>
       <c r="G29" t="n">
         <v>-0.00902915102977396</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0272086052503855</v>
+        <v>0.024763706910763</v>
       </c>
       <c r="I29" t="n">
         <v>-0.0522916142007128</v>
@@ -3452,25 +3452,25 @@
         <v>-0.140839771734219</v>
       </c>
       <c r="AA29" t="n">
-        <v>0.0742234180974693</v>
+        <v>-0.0527043427898117</v>
       </c>
       <c r="AB29" t="n">
         <v>0.104915517060876</v>
       </c>
       <c r="AC29" t="n">
-        <v>0.239056667938165</v>
+        <v>0.112269577286512</v>
       </c>
       <c r="AD29" t="n">
-        <v>0.126515032298182</v>
+        <v>-0.000412728589098861</v>
       </c>
       <c r="AE29" t="n">
         <v>0.0962839648399452</v>
       </c>
       <c r="AF29" t="n">
-        <v>-0.0677660088396269</v>
+        <v>-0.19455309949128</v>
       </c>
       <c r="AG29" t="n">
-        <v>0.250700691260953</v>
+        <v>0.156528422020213</v>
       </c>
     </row>
     <row r="30">
@@ -3490,13 +3490,13 @@
         <v>-0.186214773942108</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.16686215403164</v>
+        <v>-0.291860335754416</v>
       </c>
       <c r="G30" t="n">
         <v>-0.00871948653904214</v>
       </c>
       <c r="H30" t="n">
-        <v>0.0369848894040224</v>
+        <v>0.0345883706468194</v>
       </c>
       <c r="I30" t="n">
         <v>-0.266873947521892</v>
@@ -3553,25 +3553,25 @@
         <v>-0.139951506095078</v>
       </c>
       <c r="AA30" t="n">
-        <v>-0.398953680402588</v>
+        <v>-0.52666917896959</v>
       </c>
       <c r="AB30" t="n">
         <v>0.18995088856399</v>
       </c>
       <c r="AC30" t="n">
-        <v>-0.148199934352975</v>
+        <v>-0.275658655070582</v>
       </c>
       <c r="AD30" t="n">
-        <v>-0.132079732880696</v>
+        <v>-0.259795231447698</v>
       </c>
       <c r="AE30" t="n">
         <v>0.187576667029949</v>
       </c>
       <c r="AF30" t="n">
-        <v>-0.448390226636853</v>
+        <v>-0.575848947354461</v>
       </c>
       <c r="AG30" t="n">
-        <v>-0.115706905998653</v>
+        <v>-0.194613090461231</v>
       </c>
     </row>
     <row r="31">
@@ -3591,13 +3591,13 @@
         <v>-0.18074145350152</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.0313851804324279</v>
+        <v>-0.15535957088525</v>
       </c>
       <c r="G31" t="n">
         <v>-0.00433211445750534</v>
       </c>
       <c r="H31" t="n">
-        <v>0.043787785295544</v>
+        <v>0.0414325973251567</v>
       </c>
       <c r="I31" t="n">
         <v>-0.36382241629954</v>
@@ -3654,25 +3654,25 @@
         <v>-0.136187107329353</v>
       </c>
       <c r="AA31" t="n">
-        <v>-0.350169750618483</v>
+        <v>-0.476931589288372</v>
       </c>
       <c r="AB31" t="n">
         <v>0.0706728660628411</v>
       </c>
       <c r="AC31" t="n">
-        <v>-0.219234135309988</v>
+        <v>-0.345900938412574</v>
       </c>
       <c r="AD31" t="n">
-        <v>0.0136526656810571</v>
+        <v>-0.113109172988833</v>
       </c>
       <c r="AE31" t="n">
         <v>0.0709967202450261</v>
       </c>
       <c r="AF31" t="n">
-        <v>-0.497504370160331</v>
+        <v>-0.624171173262917</v>
       </c>
       <c r="AG31" t="n">
-        <v>-0.248286083356366</v>
+        <v>-0.353337121549218</v>
       </c>
     </row>
     <row r="32">
@@ -3692,13 +3692,13 @@
         <v>-0.188023408655981</v>
       </c>
       <c r="F32" t="n">
-        <v>0.0445220451969919</v>
+        <v>0.0910626909637126</v>
       </c>
       <c r="G32" t="n">
         <v>-0.000926599399724825</v>
       </c>
       <c r="H32" t="n">
-        <v>0.0392387337096022</v>
+        <v>0.0369153856606749</v>
       </c>
       <c r="I32" t="n">
         <v>-0.386429275379733</v>
@@ -3755,25 +3755,25 @@
         <v>-0.145161352331443</v>
       </c>
       <c r="AA32" t="n">
-        <v>-0.297987909831869</v>
+        <v>-0.253608567858958</v>
       </c>
       <c r="AB32" t="n">
         <v>0.0195130068435475</v>
       </c>
       <c r="AC32" t="n">
-        <v>-0.278413218041402</v>
+        <v>-0.23404305869826</v>
       </c>
       <c r="AD32" t="n">
-        <v>0.0884413655478634</v>
+        <v>0.132820707520774</v>
       </c>
       <c r="AE32" t="n">
         <v>0.014475621392602</v>
       </c>
       <c r="AF32" t="n">
-        <v>-0.570591322945622</v>
+        <v>-0.52622116360248</v>
       </c>
       <c r="AG32" t="n">
-        <v>-0.396062982145609</v>
+        <v>-0.480198595927784</v>
       </c>
     </row>
     <row r="33">
@@ -3793,13 +3793,13 @@
         <v>-0.184495417794735</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0625721612707403</v>
+        <v>0.128834675525228</v>
       </c>
       <c r="G33" t="n">
         <v>0.0107213802706063</v>
       </c>
       <c r="H33" t="n">
-        <v>0.0439168865394133</v>
+        <v>0.0416283220440629</v>
       </c>
       <c r="I33" t="n">
         <v>-0.42871696202656</v>
@@ -3856,25 +3856,25 @@
         <v>-0.143061358041577</v>
       </c>
       <c r="AA33" t="n">
-        <v>-0.304709825738888</v>
+        <v>-0.240484032811458</v>
       </c>
       <c r="AB33" t="n">
         <v>-0.00912811548088149</v>
       </c>
       <c r="AC33" t="n">
-        <v>-0.313867481114126</v>
+        <v>-0.249635464504215</v>
       </c>
       <c r="AD33" t="n">
-        <v>0.124007136287672</v>
+        <v>0.188232929215102</v>
       </c>
       <c r="AE33" t="n">
         <v>-0.0130690619856717</v>
       </c>
       <c r="AF33" t="n">
-        <v>-0.670358881669258</v>
+        <v>-0.606126865059347</v>
       </c>
       <c r="AG33" t="n">
-        <v>-0.546711200353016</v>
+        <v>-0.583092037319801</v>
       </c>
     </row>
     <row r="34">
@@ -3894,13 +3894,13 @@
         <v>-0.183578043716544</v>
       </c>
       <c r="F34" t="n">
-        <v>-0.0621279186476758</v>
+        <v>-0.0139896774285151</v>
       </c>
       <c r="G34" t="n">
         <v>0.00704988013781239</v>
       </c>
       <c r="H34" t="n">
-        <v>0.0255593448966518</v>
+        <v>0.0233003782332651</v>
       </c>
       <c r="I34" t="n">
         <v>-0.616876171778661</v>
@@ -3957,25 +3957,25 @@
         <v>-0.143181122174836</v>
       </c>
       <c r="AA34" t="n">
-        <v>-0.636152946721656</v>
+        <v>-0.589995381969783</v>
       </c>
       <c r="AB34" t="n">
         <v>-0.10280007135667</v>
       </c>
       <c r="AC34" t="n">
-        <v>-0.739646784072489</v>
+        <v>-0.693438933785944</v>
       </c>
       <c r="AD34" t="n">
-        <v>-0.0192767749429954</v>
+        <v>0.0268807898088781</v>
       </c>
       <c r="AE34" t="n">
         <v>-0.10280007135667</v>
       </c>
       <c r="AF34" t="n">
-        <v>-1.12836625498998</v>
+        <v>-1.08215840470343</v>
       </c>
       <c r="AG34" t="n">
-        <v>-0.716705207441297</v>
+        <v>-0.709669401657044</v>
       </c>
     </row>
   </sheetData>

</xml_diff>